<commit_message>
auto: reporte semana 2026-08-10 → 2026-08-16
</commit_message>
<xml_diff>
--- a/INFORME EXCESOS DE VELOCIDAD.xlsx
+++ b/INFORME EXCESOS DE VELOCIDAD.xlsx
@@ -222,8 +222,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SpeedingFleetsSummaryTable_1" displayName="SpeedingFleetsSummaryTable_1" ref="A5:I14" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A5:I14"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="SpeedingFleetsSummaryTable_1" displayName="SpeedingFleetsSummaryTable_1" ref="A5:I11" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A5:I11"/>
   <tableColumns count="9">
     <tableColumn id="1" name="Alias"/>
     <tableColumn id="2" name="Excesos" dataDxfId="0"/>
@@ -240,8 +240,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SpeedingFleetsDetailTable_1" displayName="SpeedingFleetsDetailTable_1" ref="A5:O27" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A5:O27"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="SpeedingFleetsDetailTable_1" displayName="SpeedingFleetsDetailTable_1" ref="A5:O20" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A5:O20"/>
   <tableColumns count="15">
     <tableColumn id="1" name="Alias"/>
     <tableColumn id="2" name="Conductor"/>
@@ -264,8 +264,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SpeedingFleetsDataTable_1" displayName="SpeedingFleetsDataTable_1" ref="A5:H59" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A5:H59"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SpeedingFleetsDataTable_1" displayName="SpeedingFleetsDataTable_1" ref="A5:H36" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A5:H36"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Alias"/>
     <tableColumn id="2" name="Secuencial" dataDxfId="0"/>
@@ -569,7 +569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30.710625" customWidth="1" style="7" min="1" max="1"/>
@@ -593,7 +593,7 @@
     <row r="3" ht="25" customHeight="1" s="8">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Desde : 2026/07/13 00:00:00 Hasta: 2026/08/08 23:59:59</t>
+          <t>Desde : 2026/07/13 00:00:00 Hasta: 2026/08/14 23:59:59</t>
         </is>
       </c>
     </row>
@@ -647,26 +647,26 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>GV TDLD-98 J PACHECHO</t>
+          <t>GLP SSZD-71  J VALLEJOS</t>
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C6" s="13" t="n">
-        <v>0.0006944444444444445</v>
+        <v>0.001840277777777778</v>
       </c>
       <c r="D6" s="13" t="n">
-        <v>0.0006944444444444445</v>
+        <v>0.0006134259259259259</v>
       </c>
       <c r="E6" s="12" t="n">
-        <v>1.6</v>
+        <v>4.1</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>100.1</v>
+        <v>104.6</v>
       </c>
       <c r="G6" s="12" t="n">
-        <v>100.1</v>
+        <v>102.2</v>
       </c>
       <c r="H6" s="12" t="n">
         <v>0</v>
@@ -678,26 +678,26 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>GV SHDV-50 C CARDENAS</t>
+          <t>GV TDLD-98 J PACHECHO</t>
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C7" s="13" t="n">
-        <v>0.001388888888888889</v>
+        <v>0.002777777777777778</v>
       </c>
       <c r="D7" s="13" t="n">
         <v>0.0006944444444444445</v>
       </c>
       <c r="E7" s="12" t="n">
-        <v>2.9</v>
+        <v>6.4</v>
       </c>
       <c r="F7" s="12" t="n">
-        <v>104.7</v>
+        <v>103.5</v>
       </c>
       <c r="G7" s="12" t="n">
-        <v>104.4</v>
+        <v>102.2</v>
       </c>
       <c r="H7" s="12" t="n">
         <v>0</v>
@@ -709,26 +709,26 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>GV TDKV-88 L CORDERO</t>
+          <t>GV SHLC-74 B MIRANDA</t>
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" s="13" t="n">
-        <v>6.944444444444444e-05</v>
+        <v>0.001388888888888889</v>
       </c>
       <c r="D8" s="13" t="n">
-        <v>6.944444444444444e-05</v>
+        <v>0.0006944444444444445</v>
       </c>
       <c r="E8" s="12" t="n">
-        <v>0.2</v>
+        <v>3</v>
       </c>
       <c r="F8" s="12" t="n">
-        <v>101.3</v>
+        <v>101.5</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>101.3</v>
+        <v>101</v>
       </c>
       <c r="H8" s="12" t="n">
         <v>0</v>
@@ -740,26 +740,26 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>GV SHLC-74 B MIRANDA</t>
+          <t>GV TM5 RXXG-15 E CABANILLA</t>
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" s="13" t="n">
-        <v>0.0006944444444444445</v>
+        <v>0.001388888888888889</v>
       </c>
       <c r="D9" s="13" t="n">
         <v>0.0006944444444444445</v>
       </c>
       <c r="E9" s="12" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="F9" s="12" t="n">
-        <v>100.5</v>
+        <v>102.8</v>
       </c>
       <c r="G9" s="12" t="n">
-        <v>100.5</v>
+        <v>102.6</v>
       </c>
       <c r="H9" s="12" t="n">
         <v>0</v>
@@ -771,26 +771,26 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>GV PEUGEOT THJY-73 J PONCE</t>
+          <t>GC TSVS-89 M AEDO</t>
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C10" s="13" t="n">
-        <v>0.0002546296296296296</v>
+        <v>0.002650462962962963</v>
       </c>
       <c r="D10" s="13" t="n">
-        <v>0.0002546296296296296</v>
+        <v>0.0008834837962962963</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>0.6</v>
+        <v>5.8</v>
       </c>
       <c r="F10" s="12" t="n">
-        <v>100.1</v>
+        <v>103.7</v>
       </c>
       <c r="G10" s="12" t="n">
-        <v>100.1</v>
+        <v>101.8</v>
       </c>
       <c r="H10" s="12" t="n">
         <v>0</v>
@@ -802,7 +802,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>GLP DF6 SRSL-99 EMERGENCIA</t>
+          <t>JAC  LYTS-17 G GALEA</t>
         </is>
       </c>
       <c r="B11" s="12" t="n">
@@ -815,111 +815,18 @@
         <v>0.0006944444444444445</v>
       </c>
       <c r="E11" s="12" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>100.8</v>
+        <v>101.1</v>
       </c>
       <c r="G11" s="12" t="n">
-        <v>100.8</v>
+        <v>101.1</v>
       </c>
       <c r="H11" s="12" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t>GLP SKDX-44 V VIAL</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="C12" s="13" t="n">
-        <v>0.002708333333333333</v>
-      </c>
-      <c r="D12" s="13" t="n">
-        <v>0.0003869097222222222</v>
-      </c>
-      <c r="E12" s="12" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="F12" s="12" t="n">
-        <v>103.6</v>
-      </c>
-      <c r="G12" s="12" t="n">
-        <v>101.7</v>
-      </c>
-      <c r="H12" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="C13" s="13" t="n">
-        <v>0.008148148148148147</v>
-      </c>
-      <c r="D13" s="13" t="n">
-        <v>0.001164016203703704</v>
-      </c>
-      <c r="E13" s="12" t="n">
-        <v>19</v>
-      </c>
-      <c r="F13" s="12" t="n">
-        <v>104</v>
-      </c>
-      <c r="G13" s="12" t="n">
-        <v>101.7</v>
-      </c>
-      <c r="H13" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>GC MAXUS PCRF-25 TERRENO</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" s="13" t="n">
-        <v>0.0006944444444444445</v>
-      </c>
-      <c r="D14" s="13" t="n">
-        <v>0.0006944444444444445</v>
-      </c>
-      <c r="E14" s="12" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F14" s="12" t="n">
-        <v>100.4</v>
-      </c>
-      <c r="G14" s="12" t="n">
-        <v>100.4</v>
-      </c>
-      <c r="H14" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -944,7 +851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O123"/>
+  <dimension ref="A1:O157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30.710625" customWidth="1" style="7" min="1" max="1"/>
@@ -972,7 +879,7 @@
     <row r="3" ht="25" customHeight="1" s="8">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Desde : 2026/07/27 00:00:00 Hasta: 2026/08/02 23:59:58</t>
+          <t>Desde : 2026/08/03 00:00:00 Hasta: 2026/08/09 23:59:58</t>
         </is>
       </c>
     </row>
@@ -7052,7 +6959,6 @@
           <t>GC TSVS-89 M AEDO</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr"/>
       <c r="C109" t="n">
         <v>1</v>
       </c>
@@ -7111,7 +7017,6 @@
           <t>GLP SSZD-71  J VALLEJOS</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr"/>
       <c r="C110" t="n">
         <v>1</v>
       </c>
@@ -7170,7 +7075,6 @@
           <t>GV TDLD-98 J PACHECHO</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr"/>
       <c r="C111" t="n">
         <v>1</v>
       </c>
@@ -7229,7 +7133,6 @@
           <t>GV SHLC-74 B MIRANDA</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr"/>
       <c r="C112" t="n">
         <v>1</v>
       </c>
@@ -7288,7 +7191,6 @@
           <t>JAC  LYTS-17 G GALEA</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr"/>
       <c r="C113" t="n">
         <v>1</v>
       </c>
@@ -7347,7 +7249,6 @@
           <t>GV SHLC-74 B MIRANDA</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr"/>
       <c r="C114" t="n">
         <v>2</v>
       </c>
@@ -7406,7 +7307,6 @@
           <t>GLP SSZD-71  J VALLEJOS</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr"/>
       <c r="C115" t="n">
         <v>2</v>
       </c>
@@ -7465,7 +7365,6 @@
           <t>GV TDLD-98 J PACHECHO</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr"/>
       <c r="C116" t="n">
         <v>2</v>
       </c>
@@ -7524,7 +7423,6 @@
           <t>GV TM5 RXXG-15 E CABANILLA</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr"/>
       <c r="C117" t="n">
         <v>1</v>
       </c>
@@ -7583,7 +7481,6 @@
           <t>GV TM5 RXXG-15 E CABANILLA</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr"/>
       <c r="C118" t="n">
         <v>2</v>
       </c>
@@ -7642,7 +7539,6 @@
           <t>GLP SSZD-71  J VALLEJOS</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr"/>
       <c r="C119" t="n">
         <v>3</v>
       </c>
@@ -7701,7 +7597,6 @@
           <t>GC TSVS-89 M AEDO</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr"/>
       <c r="C120" t="n">
         <v>2</v>
       </c>
@@ -7760,7 +7655,6 @@
           <t>GC TSVS-89 M AEDO</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr"/>
       <c r="C121" t="n">
         <v>3</v>
       </c>
@@ -7819,7 +7713,6 @@
           <t>GV TDLD-98 J PACHECHO</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr"/>
       <c r="C122" t="n">
         <v>3</v>
       </c>
@@ -7878,7 +7771,6 @@
           <t>GV TDLD-98 J PACHECHO</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr"/>
       <c r="C123" t="n">
         <v>4</v>
       </c>
@@ -7928,6 +7820,2012 @@
         <v>0</v>
       </c>
       <c r="O123" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>GV SHLC-74 B MIRANDA</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr"/>
+      <c r="C124" t="n">
+        <v>1</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>2026/08/10 09:12:32</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>-33.157548,-71.549489</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Ruta 64, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>2026/08/10 09:13:32</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>-33.165047,-71.534798</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="J124" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K124" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L124" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="M124" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="N124" t="n">
+        <v>0</v>
+      </c>
+      <c r="O124" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>GV SHDV-50 C CARDENAS</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr"/>
+      <c r="C125" t="n">
+        <v>1</v>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>2026/08/10 10:29:37</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>-32.757227,-71.420873</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Ruta 64, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>2026/08/10 10:30:38</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>-32.743513,-71.417967</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Ruta F-190, Puchuncaví, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="J125" s="14" t="n">
+        <v>0.0007060185185185185</v>
+      </c>
+      <c r="K125" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L125" t="n">
+        <v>104.2</v>
+      </c>
+      <c r="M125" t="n">
+        <v>104.2</v>
+      </c>
+      <c r="N125" t="n">
+        <v>0</v>
+      </c>
+      <c r="O125" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>GV TDLD-98 J PACHECHO</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr"/>
+      <c r="C126" t="n">
+        <v>1</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>2026/08/11 00:47:13</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>-32.977793,-71.499934</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Ruta 64, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>2026/08/11 00:48:13</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>-32.992004,-71.501153</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Ruta 64, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="J126" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K126" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L126" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="M126" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="N126" t="n">
+        <v>0</v>
+      </c>
+      <c r="O126" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>GLP SKDX-44 V VIAL</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr"/>
+      <c r="C127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>2026/08/11 01:18:36</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>-33.031585,-71.631541</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Ruta 64, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>2026/08/11 01:22:22</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>-33.031872,-71.6299</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Camino La Pólvora, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="J127" s="14" t="n">
+        <v>0.002615740740740741</v>
+      </c>
+      <c r="K127" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="L127" t="n">
+        <v>109.2</v>
+      </c>
+      <c r="M127" t="n">
+        <v>109.2</v>
+      </c>
+      <c r="N127" t="n">
+        <v>0</v>
+      </c>
+      <c r="O127" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>GV SHLC-74 B MIRANDA</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr"/>
+      <c r="C128" t="n">
+        <v>2</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>2026/08/11 09:46:56</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>-33.216008,-71.473704</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>2026/08/11 09:47:57</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>-33.229387,-71.466181</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="J128" s="14" t="n">
+        <v>0.0007060185185185185</v>
+      </c>
+      <c r="K128" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="L128" t="n">
+        <v>101</v>
+      </c>
+      <c r="M128" t="n">
+        <v>101</v>
+      </c>
+      <c r="N128" t="n">
+        <v>0</v>
+      </c>
+      <c r="O128" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>GV TDLD-98 J PACHECHO</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr"/>
+      <c r="C129" t="n">
+        <v>2</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>2026/08/11 14:25:21</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>-33.15983,-71.544708</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Ruta 64, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>2026/08/11 14:26:21</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>-33.15096,-71.557673</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+        </is>
+      </c>
+      <c r="J129" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K129" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L129" t="n">
+        <v>100.1</v>
+      </c>
+      <c r="M129" t="n">
+        <v>100.1</v>
+      </c>
+      <c r="N129" t="n">
+        <v>0</v>
+      </c>
+      <c r="O129" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>GV TDLD-98 J PACHECHO</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr"/>
+      <c r="C130" t="n">
+        <v>3</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>2026/08/11 14:48:43</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>-32.951646,-71.509458</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>2026/08/11 14:49:21</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>-32.943313,-71.513542</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Ruta E-30-F, Concón, Valparaíso, Región de Valparaíso. VMaxLiv:80, VMaxPes:80</t>
+        </is>
+      </c>
+      <c r="J130" s="14" t="n">
+        <v>0.0004398148148148148</v>
+      </c>
+      <c r="K130" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="L130" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="M130" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="N130" t="n">
+        <v>0</v>
+      </c>
+      <c r="O130" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>GLP DF6 SRSK-54 TOPOGRAFIA</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr"/>
+      <c r="C131" t="n">
+        <v>1</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>2026/08/11 15:16:59</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>-33.093469,-71.603099</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Ruta 64, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>2026/08/11 15:17:02</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>-33.094082,-71.602581</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Camino La Pólvora, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:70, VMaxPes:70</t>
+        </is>
+      </c>
+      <c r="J131" s="14" t="n">
+        <v>3.472222222222222e-05</v>
+      </c>
+      <c r="K131" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L131" t="n">
+        <v>104.6</v>
+      </c>
+      <c r="M131" t="n">
+        <v>104.6</v>
+      </c>
+      <c r="N131" t="n">
+        <v>0</v>
+      </c>
+      <c r="O131" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>GC MAXUS PKFF-65 G VICENCIO</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr"/>
+      <c r="C132" t="n">
+        <v>1</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>2026/08/11 17:10:00</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>-32.798908,-71.440814</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>Ruta 64, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>2026/08/11 17:11:00</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>-32.810983,-71.441434</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Ruta F-190, Quintero, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="J132" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K132" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="L132" t="n">
+        <v>107.1</v>
+      </c>
+      <c r="M132" t="n">
+        <v>107.1</v>
+      </c>
+      <c r="N132" t="n">
+        <v>0</v>
+      </c>
+      <c r="O132" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>GC MAXUS PKFF-65 G VICENCIO</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr"/>
+      <c r="C133" t="n">
+        <v>2</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>2026/08/11 17:31:29</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>-32.942137,-71.482014</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>Ruta F-190, Quintero, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>2026/08/11 17:32:08</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>-32.9487,-71.483747</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Ruta 64, Concón, Valparaíso, Región de Valparaíso. VMaxLiv:70, VMaxPes:70</t>
+        </is>
+      </c>
+      <c r="J133" s="14" t="n">
+        <v>0.0004513888888888889</v>
+      </c>
+      <c r="K133" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L133" t="n">
+        <v>104</v>
+      </c>
+      <c r="M133" t="n">
+        <v>104</v>
+      </c>
+      <c r="N133" t="n">
+        <v>0</v>
+      </c>
+      <c r="O133" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>GV SHLC-74 B MIRANDA</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr"/>
+      <c r="C134" t="n">
+        <v>3</v>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>2026/08/11 22:16:04</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>-33.217343,-71.472838</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>2026/08/11 22:17:04</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>-33.205626,-71.484055</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+        </is>
+      </c>
+      <c r="J134" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K134" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L134" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="M134" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="N134" t="n">
+        <v>0</v>
+      </c>
+      <c r="O134" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>GC MAXUS PKFF-65 G VICENCIO</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr"/>
+      <c r="C135" t="n">
+        <v>3</v>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>2026/08/12 11:16:15</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>-33.38297,-71.391372</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Ruta 64, Concón, Valparaíso, Región de Valparaíso. VMaxLiv:70, VMaxPes:70</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>2026/08/12 11:17:15</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>-33.396877,-71.394671</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Ruta F-74-G, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:60, VMaxPes:60</t>
+        </is>
+      </c>
+      <c r="J135" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K135" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L135" t="n">
+        <v>102.1</v>
+      </c>
+      <c r="M135" t="n">
+        <v>102.1</v>
+      </c>
+      <c r="N135" t="n">
+        <v>0</v>
+      </c>
+      <c r="O135" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>GLP SKDX-44 V VIAL</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr"/>
+      <c r="C136" t="n">
+        <v>2</v>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>2026/08/12 12:27:11</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>-33.113036,-71.560164</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>Camino La Pólvora, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>2026/08/12 12:27:50</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>-33.121189,-71.561416</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>s/n, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="J136" s="14" t="n">
+        <v>0.0004513888888888889</v>
+      </c>
+      <c r="K136" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="L136" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="M136" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="N136" t="n">
+        <v>0</v>
+      </c>
+      <c r="O136" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>GV TDLD-98 J PACHECHO</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr"/>
+      <c r="C137" t="n">
+        <v>4</v>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>2026/08/12 14:44:39</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>-33.163382,-71.537721</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Ruta E-30-F, Concón, Valparaíso, Región de Valparaíso. VMaxLiv:80, VMaxPes:80</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>2026/08/12 14:45:39</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>-33.155922,-71.552342</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+        </is>
+      </c>
+      <c r="J137" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K137" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L137" t="n">
+        <v>100.3</v>
+      </c>
+      <c r="M137" t="n">
+        <v>100.3</v>
+      </c>
+      <c r="N137" t="n">
+        <v>0</v>
+      </c>
+      <c r="O137" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>GV TDLD-98 J PACHECHO</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr"/>
+      <c r="C138" t="n">
+        <v>5</v>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>2026/08/12 14:47:39</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>-33.13014,-71.561957</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>2026/08/12 14:48:39</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>-33.115708,-71.560383</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+        </is>
+      </c>
+      <c r="J138" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K138" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L138" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="M138" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="N138" t="n">
+        <v>0</v>
+      </c>
+      <c r="O138" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>GC MAXUS PKFF-65 G VICENCIO</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr"/>
+      <c r="C139" t="n">
+        <v>4</v>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>2026/08/12 15:55:12</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>-33.376179,-71.386332</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>Ruta F-74-G, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:60, VMaxPes:60</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>2026/08/12 15:55:25</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>-33.373618,-71.385271</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Ruta F-74-G, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:60, VMaxPes:60</t>
+        </is>
+      </c>
+      <c r="J139" s="14" t="n">
+        <v>0.000150462962962963</v>
+      </c>
+      <c r="K139" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="L139" t="n">
+        <v>102.6</v>
+      </c>
+      <c r="M139" t="n">
+        <v>102.6</v>
+      </c>
+      <c r="N139" t="n">
+        <v>0</v>
+      </c>
+      <c r="O139" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>GC MAXUS PKFF-65 G VICENCIO</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr"/>
+      <c r="C140" t="n">
+        <v>5</v>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>2026/08/12 16:13:58</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>-33.305002,-71.411287</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Ruta F-74-G, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:60, VMaxPes:60</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>2026/08/12 16:15:57</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>-33.277849,-71.428907</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="J140" s="14" t="n">
+        <v>0.001377314814814815</v>
+      </c>
+      <c r="K140" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="L140" t="n">
+        <v>108.6</v>
+      </c>
+      <c r="M140" t="n">
+        <v>107.3</v>
+      </c>
+      <c r="N140" t="n">
+        <v>0</v>
+      </c>
+      <c r="O140" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>GC MAXUS PKFF-65 G VICENCIO</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr"/>
+      <c r="C141" t="n">
+        <v>6</v>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>2026/08/12 17:29:08</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>-32.982117,-71.500227</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>2026/08/12 17:29:59</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>-32.970275,-71.5001</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Ruta E-30-F, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:80, VMaxPes:80</t>
+        </is>
+      </c>
+      <c r="J141" s="14" t="n">
+        <v>0.0005902777777777778</v>
+      </c>
+      <c r="K141" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="L141" t="n">
+        <v>107</v>
+      </c>
+      <c r="M141" t="n">
+        <v>107</v>
+      </c>
+      <c r="N141" t="n">
+        <v>0</v>
+      </c>
+      <c r="O141" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>GC MAXUS PKFF-65 G VICENCIO</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr"/>
+      <c r="C142" t="n">
+        <v>7</v>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>2026/08/12 17:32:09</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>-32.943489,-71.513534</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>Ruta E-30-F, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:80, VMaxPes:80</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>2026/08/12 17:33:09</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>-32.929667,-71.512068</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Ruta E-30-F, Concón, Valparaíso, Región de Valparaíso. VMaxLiv:80, VMaxPes:80</t>
+        </is>
+      </c>
+      <c r="J142" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K142" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L142" t="n">
+        <v>110.7</v>
+      </c>
+      <c r="M142" t="n">
+        <v>110.7</v>
+      </c>
+      <c r="N142" t="n">
+        <v>0</v>
+      </c>
+      <c r="O142" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>GV PEUGEOT THJY-73 J PONCE</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr"/>
+      <c r="C143" t="n">
+        <v>1</v>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>2026/08/13 07:27:21</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>-33.054539,-71.335674</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Ruta 64, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>2026/08/13 07:28:21</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>-33.063291,-71.348177</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Autopista Troncal Sur, Villa Alemana, Marga Marga, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="J143" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K143" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L143" t="n">
+        <v>100.3</v>
+      </c>
+      <c r="M143" t="n">
+        <v>100.3</v>
+      </c>
+      <c r="N143" t="n">
+        <v>0</v>
+      </c>
+      <c r="O143" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>GV PEUGEOT THJY-73 J PONCE</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr"/>
+      <c r="C144" t="n">
+        <v>2</v>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>2026/08/13 09:17:07</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>-33.09653,-71.545845</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Autopista Troncal Sur, Villa Alemana, Marga Marga, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>2026/08/13 09:17:46</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>-33.088266,-71.5422</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Vía Las Palmas, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:80, VMaxPes:80</t>
+        </is>
+      </c>
+      <c r="J144" s="14" t="n">
+        <v>0.0004513888888888889</v>
+      </c>
+      <c r="K144" t="n">
+        <v>1</v>
+      </c>
+      <c r="L144" t="n">
+        <v>100.6</v>
+      </c>
+      <c r="M144" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="N144" t="n">
+        <v>0</v>
+      </c>
+      <c r="O144" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>GC MAXUS PKFF-65 G VICENCIO</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr"/>
+      <c r="C145" t="n">
+        <v>8</v>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>2026/08/13 09:24:35</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>-32.985661,-71.500562</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>Ruta E-30-F, Concón, Valparaíso, Región de Valparaíso. VMaxLiv:80, VMaxPes:80</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>2026/08/13 09:25:32</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>-32.998254,-71.502383</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Camino Internacional Valparaíso - Mendoza, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+        </is>
+      </c>
+      <c r="J145" s="14" t="n">
+        <v>0.0006597222222222222</v>
+      </c>
+      <c r="K145" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="L145" t="n">
+        <v>107.7</v>
+      </c>
+      <c r="M145" t="n">
+        <v>107.7</v>
+      </c>
+      <c r="N145" t="n">
+        <v>0</v>
+      </c>
+      <c r="O145" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>GV SHLC-74 B MIRANDA</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr"/>
+      <c r="C146" t="n">
+        <v>4</v>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>2026/08/13 10:02:31</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>-33.35848,-71.326553</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>2026/08/13 10:03:31</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>-33.364972,-71.312258</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="J146" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K146" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="L146" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="M146" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="N146" t="n">
+        <v>0</v>
+      </c>
+      <c r="O146" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>GV SHDV-50 C CARDENAS</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr"/>
+      <c r="C147" t="n">
+        <v>2</v>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>2026/08/13 10:39:59</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>-33.227,-71.467768</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>Ruta F-190, Puchuncaví, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>2026/08/13 10:40:59</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>-33.213935,-71.475097</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="J147" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K147" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L147" t="n">
+        <v>108</v>
+      </c>
+      <c r="M147" t="n">
+        <v>108</v>
+      </c>
+      <c r="N147" t="n">
+        <v>0</v>
+      </c>
+      <c r="O147" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>GV SHDV-50 C CARDENAS</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr"/>
+      <c r="C148" t="n">
+        <v>3</v>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>2026/08/13 10:49:59</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>-33.119158,-71.56076</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>2026/08/13 10:50:42</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>-33.109677,-71.558209</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+        </is>
+      </c>
+      <c r="J148" s="14" t="n">
+        <v>0.0004976851851851852</v>
+      </c>
+      <c r="K148" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="L148" t="n">
+        <v>108.5</v>
+      </c>
+      <c r="M148" t="n">
+        <v>108.5</v>
+      </c>
+      <c r="N148" t="n">
+        <v>0</v>
+      </c>
+      <c r="O148" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>JAC  LYTS-17 G GALEA</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr"/>
+      <c r="C149" t="n">
+        <v>1</v>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>2026/08/13 11:57:49</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>-33.285524,-71.411366</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Ruta 64, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>2026/08/13 11:58:27</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>-33.279484,-71.413704</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Ruta F-852, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="J149" s="14" t="n">
+        <v>0.0004398148148148148</v>
+      </c>
+      <c r="K149" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="L149" t="n">
+        <v>107.6</v>
+      </c>
+      <c r="M149" t="n">
+        <v>107.6</v>
+      </c>
+      <c r="N149" t="n">
+        <v>0</v>
+      </c>
+      <c r="O149" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>GV TDLD-98 J PACHECHO</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr"/>
+      <c r="C150" t="n">
+        <v>6</v>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>2026/08/13 14:31:13</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>-33.225857,-71.468365</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>2026/08/13 14:32:13</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>-33.213027,-71.475997</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="J150" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K150" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L150" t="n">
+        <v>100.3</v>
+      </c>
+      <c r="M150" t="n">
+        <v>100.3</v>
+      </c>
+      <c r="N150" t="n">
+        <v>0</v>
+      </c>
+      <c r="O150" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>GV SHDV-50 C CARDENAS</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr"/>
+      <c r="C151" t="n">
+        <v>4</v>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>2026/08/13 18:25:02</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>-33.268542,-71.432855</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>2026/08/13 18:26:02</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>-33.255908,-71.44039</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+        </is>
+      </c>
+      <c r="J151" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K151" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L151" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="M151" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="N151" t="n">
+        <v>0</v>
+      </c>
+      <c r="O151" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>GV SHDV-50 C CARDENAS</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr"/>
+      <c r="C152" t="n">
+        <v>5</v>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>2026/08/13 18:48:02</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>-33.071993,-71.571936</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>2026/08/13 18:48:57</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>-33.063353,-71.582457</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>José Santos Ossa, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:80, VMaxPes:80</t>
+        </is>
+      </c>
+      <c r="J152" s="14" t="n">
+        <v>0.0006365740740740741</v>
+      </c>
+      <c r="K152" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="L152" t="n">
+        <v>109.5</v>
+      </c>
+      <c r="M152" t="n">
+        <v>109.5</v>
+      </c>
+      <c r="N152" t="n">
+        <v>0</v>
+      </c>
+      <c r="O152" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>GV SHLC-74 B MIRANDA</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr"/>
+      <c r="C153" t="n">
+        <v>5</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>2026/08/13 22:23:11</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>-33.203884,-71.485888</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>2026/08/13 22:24:11</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>-33.192111,-71.496379</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="J153" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K153" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="L153" t="n">
+        <v>102.1</v>
+      </c>
+      <c r="M153" t="n">
+        <v>102.1</v>
+      </c>
+      <c r="N153" t="n">
+        <v>0</v>
+      </c>
+      <c r="O153" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>GV TDLD-98 J PACHECHO</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr"/>
+      <c r="C154" t="n">
+        <v>7</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>2026/08/14 00:38:07</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>-32.98055,-71.500149</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>2026/08/14 00:39:07</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>-32.994359,-71.501297</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>Ruta 64, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="J154" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K154" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L154" t="n">
+        <v>100.2</v>
+      </c>
+      <c r="M154" t="n">
+        <v>100.2</v>
+      </c>
+      <c r="N154" t="n">
+        <v>0</v>
+      </c>
+      <c r="O154" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>GV SHDV-50 C CARDENAS</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr"/>
+      <c r="C155" t="n">
+        <v>6</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>2026/08/14 08:05:03</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>-33.10634,-71.549378</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>José Santos Ossa, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:80, VMaxPes:80</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>2026/08/14 08:05:51</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>-33.112291,-71.560068</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+        </is>
+      </c>
+      <c r="J155" s="14" t="n">
+        <v>0.0005555555555555556</v>
+      </c>
+      <c r="K155" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="L155" t="n">
+        <v>108.7</v>
+      </c>
+      <c r="M155" t="n">
+        <v>107.7</v>
+      </c>
+      <c r="N155" t="n">
+        <v>0</v>
+      </c>
+      <c r="O155" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>GC TSVS-89 M AEDO</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr"/>
+      <c r="C156" t="n">
+        <v>1</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>2026/08/14 19:10:37</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>-33.053836,-71.334523</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>Ruta 64, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>2026/08/14 19:11:38</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>-33.063285,-71.348089</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Autopista Troncal Sur, Villa Alemana, Marga Marga, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="J156" s="14" t="n">
+        <v>0.0007060185185185185</v>
+      </c>
+      <c r="K156" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L156" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="M156" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="N156" t="n">
+        <v>0</v>
+      </c>
+      <c r="O156" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>GC TSVS-89 M AEDO</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr"/>
+      <c r="C157" t="n">
+        <v>2</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>2026/08/14 19:12:38</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>-33.06932,-71.363576</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>Autopista Troncal Sur, Villa Alemana, Marga Marga, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>2026/08/14 19:13:38</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>-33.067875,-71.380877</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Autopista Troncal Sur, Villa Alemana, Marga Marga, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+        </is>
+      </c>
+      <c r="J157" s="14" t="n">
+        <v>0.0006944444444444445</v>
+      </c>
+      <c r="K157" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="L157" t="n">
+        <v>101.3</v>
+      </c>
+      <c r="M157" t="n">
+        <v>101.3</v>
+      </c>
+      <c r="N157" t="n">
+        <v>0</v>
+      </c>
+      <c r="O157" t="n">
         <v>0</v>
       </c>
     </row>
@@ -7952,7 +9850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30.710625" customWidth="1" style="7" min="1" max="1"/>
@@ -7978,7 +9876,7 @@
     <row r="3" ht="25" customHeight="1" s="8">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Desde : 2026/07/27 00:00:00 Hasta: 2026/08/02 23:59:58</t>
+          <t>Desde : 2026/08/03 00:00:00 Hasta: 2026/08/09 23:59:58</t>
         </is>
       </c>
     </row>
@@ -8027,7 +9925,7 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>GV TDLD-98 J PACHECHO</t>
+          <t>GLP SSZD-71  J VALLEJOS</t>
         </is>
       </c>
       <c r="B6" s="12" t="n">
@@ -8035,33 +9933,33 @@
       </c>
       <c r="C6" s="12" t="inlineStr">
         <is>
-          <t>2026/08/02 14:32:36</t>
+          <t>2026/08/05 12:23:39</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>-33.16243,-71.539564</t>
+          <t>-33.080686,-71.561833</t>
         </is>
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+          <t>José Santos Ossa, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
         </is>
       </c>
       <c r="F6" s="12" t="n">
-        <v>100.1</v>
+        <v>104.6</v>
       </c>
       <c r="G6" s="12" t="n">
-        <v>77880.5</v>
+        <v>61389.2</v>
       </c>
       <c r="H6" s="12" t="n">
-        <v>360.8</v>
+        <v>176.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>GV TDLD-98 J PACHECHO</t>
+          <t>GLP SSZD-71  J VALLEJOS</t>
         </is>
       </c>
       <c r="B7" s="12" t="n">
@@ -8069,169 +9967,169 @@
       </c>
       <c r="C7" s="12" t="inlineStr">
         <is>
-          <t>2026/08/02 14:33:36</t>
+          <t>2026/08/05 12:24:39</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>-33.15517,-71.553769</t>
+          <t>-33.070089,-71.574806</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+          <t>José Santos Ossa, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
         </is>
       </c>
       <c r="F7" s="12" t="n">
-        <v>91.2</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="G7" s="12" t="n">
-        <v>77882.10000000001</v>
+        <v>61390.9</v>
       </c>
       <c r="H7" s="12" t="n">
-        <v>356.3</v>
+        <v>162</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>GV SHDV-50 C CARDENAS</t>
+          <t>GLP SSZD-71  J VALLEJOS</t>
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" s="12" t="inlineStr">
         <is>
-          <t>2026/07/30 18:54:20</t>
+          <t>2026/08/06 12:13:09</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>-32.897768,-71.449538</t>
+          <t>-33.059575,-71.530514</t>
         </is>
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>Ruta F-190, Quillota, Quillota, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+          <t>Ruta Las Palmas, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
         </is>
       </c>
       <c r="F8" s="12" t="n">
-        <v>104.7</v>
+        <v>101.7</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>187456</v>
+        <v>61506.4</v>
       </c>
       <c r="H8" s="12" t="n">
-        <v>125.6</v>
+        <v>267.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>GV SHDV-50 C CARDENAS</t>
+          <t>GLP SSZD-71  J VALLEJOS</t>
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>2026/07/30 18:55:20</t>
+          <t>2026/08/06 12:13:48</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>-32.906604,-71.440511</t>
+          <t>-33.066788,-71.533562</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>Ruta F-190, Quillota, Quillota, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+          <t>Ruta Las Palmas, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
         </is>
       </c>
       <c r="F9" s="12" t="n">
-        <v>76.7</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="G9" s="12" t="n">
-        <v>187457.3</v>
+        <v>61507.3</v>
       </c>
       <c r="H9" s="12" t="n">
-        <v>124.3</v>
+        <v>305.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>GV SHDV-50 C CARDENAS</t>
+          <t>GLP SSZD-71  J VALLEJOS</t>
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>2026/07/31 13:08:39</t>
+          <t>2026/08/07 12:07:15</t>
         </is>
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>-33.219324,-71.471926</t>
+          <t>-33.094897,-71.600273</t>
         </is>
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+          <t>Camino La Pólvora, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:70, VMaxPes:70</t>
         </is>
       </c>
       <c r="F10" s="12" t="n">
-        <v>104.1</v>
+        <v>100.2</v>
       </c>
       <c r="G10" s="12" t="n">
-        <v>187526.8</v>
+        <v>61623.8</v>
       </c>
       <c r="H10" s="12" t="n">
-        <v>330.6</v>
+        <v>427.8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>GV SHDV-50 C CARDENAS</t>
+          <t>GLP SSZD-71  J VALLEJOS</t>
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>2026/07/31 13:09:39</t>
+          <t>2026/08/07 12:08:15</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>-33.231962,-71.464083</t>
+          <t>-33.089443,-71.614598</t>
         </is>
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
+          <t>Camino La Pólvora, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:70, VMaxPes:70</t>
         </is>
       </c>
       <c r="F11" s="12" t="n">
-        <v>94.7</v>
+        <v>84</v>
       </c>
       <c r="G11" s="12" t="n">
-        <v>187528.4</v>
+        <v>61625.3</v>
       </c>
       <c r="H11" s="12" t="n">
-        <v>337.4</v>
+        <v>469.4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>GV TDKV-88 L CORDERO</t>
+          <t>GV TDLD-98 J PACHECHO</t>
         </is>
       </c>
       <c r="B12" s="12" t="n">
@@ -8239,12 +10137,12 @@
       </c>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>2026/07/30 17:56:03</t>
+          <t>2026/08/05 14:23:46</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
         <is>
-          <t>-33.10693,-71.550214</t>
+          <t>-33.163504,-71.537483</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
@@ -8253,19 +10151,19 @@
         </is>
       </c>
       <c r="F12" s="12" t="n">
-        <v>101.3</v>
+        <v>101</v>
       </c>
       <c r="G12" s="12" t="n">
-        <v>76539</v>
+        <v>78551.10000000001</v>
       </c>
       <c r="H12" s="12" t="n">
-        <v>351.1</v>
+        <v>367.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>GV TDKV-88 L CORDERO</t>
+          <t>GV TDLD-98 J PACHECHO</t>
         </is>
       </c>
       <c r="B13" s="12" t="n">
@@ -8273,12 +10171,12 @@
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>2026/07/30 17:56:09</t>
+          <t>2026/08/05 14:24:46</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>-33.107497,-71.5518</t>
+          <t>-33.156097,-71.552015</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
@@ -8287,223 +10185,223 @@
         </is>
       </c>
       <c r="F13" s="12" t="n">
-        <v>93.2</v>
+        <v>93</v>
       </c>
       <c r="G13" s="12" t="n">
-        <v>76539.2</v>
+        <v>78552.7</v>
       </c>
       <c r="H13" s="12" t="n">
-        <v>347.1</v>
+        <v>368.1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>GV SHLC-74 B MIRANDA</t>
+          <t>GV TDLD-98 J PACHECHO</t>
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C14" s="12" t="inlineStr">
         <is>
-          <t>2026/07/31 07:36:59</t>
+          <t>2026/08/06 14:22:56</t>
         </is>
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>-33.158797,-71.546799</t>
+          <t>-33.231385,-71.464327</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
         </is>
       </c>
       <c r="F14" s="12" t="n">
-        <v>100.5</v>
+        <v>100.8</v>
       </c>
       <c r="G14" s="12" t="n">
-        <v>122625.2</v>
+        <v>78768</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>369.3</v>
+        <v>340</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>GV SHLC-74 B MIRANDA</t>
+          <t>GV TDLD-98 J PACHECHO</t>
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>2026/07/31 07:37:59</t>
+          <t>2026/08/06 14:23:56</t>
         </is>
       </c>
       <c r="D15" s="15" t="inlineStr">
         <is>
-          <t>-33.149438,-71.558461</t>
+          <t>-33.219271,-71.471768</t>
         </is>
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
         </is>
       </c>
       <c r="F15" s="12" t="n">
-        <v>89.90000000000001</v>
+        <v>85.7</v>
       </c>
       <c r="G15" s="12" t="n">
-        <v>122626.7</v>
+        <v>78769.5</v>
       </c>
       <c r="H15" s="12" t="n">
-        <v>344.9</v>
+        <v>335.5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>GV PEUGEOT THJY-73 J PONCE</t>
+          <t>GV TDLD-98 J PACHECHO</t>
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C16" s="12" t="inlineStr">
         <is>
-          <t>2026/07/28 15:58:20</t>
+          <t>2026/08/08 01:32:10</t>
         </is>
       </c>
       <c r="D16" s="15" t="inlineStr">
         <is>
-          <t>-32.733776,-71.436634</t>
+          <t>-33.234063,-71.462269</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Ruta F-20, Puchuncaví, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
         </is>
       </c>
       <c r="F16" s="12" t="n">
-        <v>100.1</v>
+        <v>103.3</v>
       </c>
       <c r="G16" s="12" t="n">
-        <v>122447.9</v>
+        <v>79183.89999999999</v>
       </c>
       <c r="H16" s="12" t="n">
-        <v>26.1</v>
+        <v>344</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>GV PEUGEOT THJY-73 J PONCE</t>
+          <t>GV TDLD-98 J PACHECHO</t>
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>2026/07/28 15:58:42</t>
+          <t>2026/08/08 01:33:10</t>
         </is>
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>-32.736051,-71.431128</t>
+          <t>-33.244036,-71.449798</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Ruta F-20, Puchuncaví, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
         </is>
       </c>
       <c r="F17" s="12" t="n">
-        <v>93</v>
+        <v>98.2</v>
       </c>
       <c r="G17" s="12" t="n">
-        <v>122448.5</v>
+        <v>79185.5</v>
       </c>
       <c r="H17" s="12" t="n">
-        <v>16.5</v>
+        <v>276.9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>GLP DF6 SRSL-99 EMERGENCIA</t>
+          <t>GV TDLD-98 J PACHECHO</t>
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>2026/07/28 02:11:25</t>
+          <t>2026/08/08 14:19:07</t>
         </is>
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>-32.944023,-71.513376</t>
+          <t>-33.232909,-71.463096</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Ruta E-30-F, Concón, Valparaíso, Región de Valparaíso. VMaxLiv:80, VMaxPes:80</t>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
         </is>
       </c>
       <c r="F18" s="12" t="n">
-        <v>100.8</v>
+        <v>103.5</v>
       </c>
       <c r="G18" s="12" t="n">
-        <v>261970.6</v>
+        <v>79225.7</v>
       </c>
       <c r="H18" s="12" t="n">
-        <v>123</v>
+        <v>345.6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>GLP DF6 SRSL-99 EMERGENCIA</t>
+          <t>GV TDLD-98 J PACHECHO</t>
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>2026/07/28 02:12:25</t>
+          <t>2026/08/08 14:20:07</t>
         </is>
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>-32.935778,-71.513703</t>
+          <t>-33.219807,-71.471478</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Ruta E-30-F, Concón, Valparaíso, Región de Valparaíso. VMaxLiv:80, VMaxPes:80</t>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
         </is>
       </c>
       <c r="F19" s="12" t="n">
-        <v>0</v>
+        <v>90.2</v>
       </c>
       <c r="G19" s="12" t="n">
-        <v>261971.5</v>
+        <v>79227.39999999999</v>
       </c>
       <c r="H19" s="12" t="n">
-        <v>84.90000000000001</v>
+        <v>336.1</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>GV SHLC-74 B MIRANDA</t>
         </is>
       </c>
       <c r="B20" s="12" t="n">
@@ -8511,33 +10409,33 @@
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 06:30:23</t>
+          <t>2026/08/05 16:09:19</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>-33.102452,-71.54806</t>
+          <t>-32.786803,-71.431676</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+          <t>Ruta F-190, Quintero, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
         </is>
       </c>
       <c r="F20" s="12" t="n">
-        <v>102.1</v>
+        <v>101.5</v>
       </c>
       <c r="G20" s="12" t="n">
-        <v>147132</v>
+        <v>124111.7</v>
       </c>
       <c r="H20" s="12" t="n">
-        <v>345.3</v>
+        <v>67.40000000000001</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>GV SHLC-74 B MIRANDA</t>
         </is>
       </c>
       <c r="B21" s="12" t="n">
@@ -8545,33 +10443,33 @@
       </c>
       <c r="C21" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 06:30:48</t>
+          <t>2026/08/05 16:10:19</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>-33.096687,-71.546062</t>
+          <t>-32.797308,-71.44036</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>s/n, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:80, VMaxPes:80</t>
+          <t>Ruta F-190, Quintero, Valparaíso, Región de Valparaíso. VMaxLiv:70, VMaxPes:70</t>
         </is>
       </c>
       <c r="F21" s="12" t="n">
-        <v>95.90000000000001</v>
+        <v>97.8</v>
       </c>
       <c r="G21" s="12" t="n">
-        <v>147132.7</v>
+        <v>124113.1</v>
       </c>
       <c r="H21" s="12" t="n">
-        <v>310.4</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>GV SHLC-74 B MIRANDA</t>
         </is>
       </c>
       <c r="B22" s="12" t="n">
@@ -8579,33 +10477,33 @@
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 06:46:24</t>
+          <t>2026/08/06 09:46:47</t>
         </is>
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>-32.967111,-71.503823</t>
+          <t>-33.205819,-71.48396</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Ruta E-30-F, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:80, VMaxPes:80</t>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
         </is>
       </c>
       <c r="F22" s="12" t="n">
-        <v>102.6</v>
+        <v>100.5</v>
       </c>
       <c r="G22" s="12" t="n">
-        <v>147153.7</v>
+        <v>124379.3</v>
       </c>
       <c r="H22" s="12" t="n">
-        <v>159.9</v>
+        <v>400</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>GV SHLC-74 B MIRANDA</t>
         </is>
       </c>
       <c r="B23" s="12" t="n">
@@ -8613,1251 +10511,469 @@
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 06:47:14</t>
+          <t>2026/08/06 09:47:47</t>
         </is>
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>-32.957174,-71.510191</t>
+          <t>-33.216959,-71.473175</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr">
         <is>
-          <t>Ruta E-30-F, Concón, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
         </is>
       </c>
       <c r="F23" s="12" t="n">
-        <v>88.8</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="G23" s="12" t="n">
-        <v>147155</v>
+        <v>124380.9</v>
       </c>
       <c r="H23" s="12" t="n">
-        <v>171.1</v>
+        <v>335.6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>GV TM5 RXXG-15 E CABANILLA</t>
         </is>
       </c>
       <c r="B24" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 06:50:24</t>
+          <t>2026/08/07 07:01:46</t>
         </is>
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>-32.989287,-71.500906</t>
+          <t>-33.275515,-71.429868</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
         <is>
-          <t>Camino Internacional, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
         </is>
       </c>
       <c r="F24" s="12" t="n">
-        <v>103.1</v>
+        <v>102.3</v>
       </c>
       <c r="G24" s="12" t="n">
-        <v>147159.5</v>
+        <v>22879</v>
       </c>
       <c r="H24" s="12" t="n">
-        <v>136.8</v>
+        <v>298.5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>GV TM5 RXXG-15 E CABANILLA</t>
         </is>
       </c>
       <c r="B25" s="12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 06:51:02</t>
+          <t>2026/08/07 07:02:46</t>
         </is>
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
-          <t>-32.998137,-71.50228</t>
+          <t>-33.262462,-71.43552</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>Camino Internacional, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+          <t>Ruta 68, Casablanca, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
         </is>
       </c>
       <c r="F25" s="12" t="n">
-        <v>80</v>
+        <v>91.8</v>
       </c>
       <c r="G25" s="12" t="n">
-        <v>147160.4</v>
+        <v>22880.5</v>
       </c>
       <c r="H25" s="12" t="n">
-        <v>153.9</v>
+        <v>291</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>GV TM5 RXXG-15 E CABANILLA</t>
         </is>
       </c>
       <c r="B26" s="12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 09:40:00</t>
+          <t>2026/08/07 07:14:46</t>
         </is>
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
-          <t>-33.013677,-71.500475</t>
+          <t>-33.143468,-71.561375</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
         <is>
-          <t>Avenida Carlos Ibáñez del Campo, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:70, VMaxPes:70</t>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
         </is>
       </c>
       <c r="F26" s="12" t="n">
-        <v>100.4</v>
+        <v>102.8</v>
       </c>
       <c r="G26" s="12" t="n">
-        <v>147253.8</v>
+        <v>22898.6</v>
       </c>
       <c r="H26" s="12" t="n">
-        <v>249.7</v>
+        <v>331.1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>GV TM5 RXXG-15 E CABANILLA</t>
         </is>
       </c>
       <c r="B27" s="12" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 09:40:16</t>
+          <t>2026/08/07 07:15:46</t>
         </is>
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
-          <t>-33.017375,-71.500179</t>
+          <t>-33.130053,-71.561948</t>
         </is>
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Avenida Rubén Hurtado, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:70, VMaxPes:70</t>
+          <t>Ruta 68, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
         </is>
       </c>
       <c r="F27" s="12" t="n">
-        <v>93.3</v>
+        <v>87.7</v>
       </c>
       <c r="G27" s="12" t="n">
-        <v>147254.2</v>
+        <v>22900.1</v>
       </c>
       <c r="H27" s="12" t="n">
-        <v>240.3</v>
+        <v>336</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>GC TSVS-89 M AEDO</t>
         </is>
       </c>
       <c r="B28" s="12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C28" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 11:31:13</t>
+          <t>2026/08/03 06:01:10</t>
         </is>
       </c>
       <c r="D28" s="15" t="inlineStr">
         <is>
-          <t>-33.059472,-71.645814</t>
+          <t>-33.063154,-71.469437</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
         <is>
-          <t>Camino La Pólvora, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:60, VMaxPes:60</t>
+          <t>Autopista Troncal Sur, Quilpué, Marga Marga, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
         </is>
       </c>
       <c r="F28" s="12" t="n">
-        <v>100.6</v>
+        <v>100.2</v>
       </c>
       <c r="G28" s="12" t="n">
-        <v>147292.5</v>
+        <v>117052.1</v>
       </c>
       <c r="H28" s="12" t="n">
-        <v>322.9</v>
+        <v>116.8</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>GC TSVS-89 M AEDO</t>
         </is>
       </c>
       <c r="B29" s="12" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C29" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 11:31:21</t>
+          <t>2026/08/03 06:02:10</t>
         </is>
       </c>
       <c r="D29" s="15" t="inlineStr">
         <is>
-          <t>-33.060679,-71.644303</t>
+          <t>-33.061893,-71.457259</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Camino La Pólvora, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:60, VMaxPes:60</t>
+          <t>s/n, Quilpué, Marga Marga, Región de Valparaíso. VMaxLiv:60, VMaxPes:60</t>
         </is>
       </c>
       <c r="F29" s="12" t="n">
-        <v>89.59999999999999</v>
+        <v>29.7</v>
       </c>
       <c r="G29" s="12" t="n">
-        <v>147292.8</v>
+        <v>117053.3</v>
       </c>
       <c r="H29" s="12" t="n">
-        <v>335.3</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>GC TSVS-89 M AEDO</t>
         </is>
       </c>
       <c r="B30" s="12" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 11:31:50</t>
+          <t>2026/08/07 18:21:12</t>
         </is>
       </c>
       <c r="D30" s="15" t="inlineStr">
         <is>
-          <t>-33.06623,-71.64223</t>
+          <t>-32.924007,-71.28105</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
         <is>
-          <t>Camino La Pólvora, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:60, VMaxPes:60</t>
+          <t>Autopista Los Andes, Quillota, Quillota, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
         </is>
       </c>
       <c r="F30" s="12" t="n">
-        <v>101.2</v>
+        <v>101.6</v>
       </c>
       <c r="G30" s="12" t="n">
-        <v>147293.5</v>
+        <v>118469.3</v>
       </c>
       <c r="H30" s="12" t="n">
-        <v>386.3</v>
+        <v>85.5</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>GC TSVS-89 M AEDO</t>
         </is>
       </c>
       <c r="B31" s="12" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C31" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 11:31:55</t>
+          <t>2026/08/07 18:22:01</t>
         </is>
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>-33.067011,-71.641101</t>
+          <t>-32.933575,-71.288625</t>
         </is>
       </c>
       <c r="E31" s="12" t="inlineStr">
         <is>
-          <t>Camino La Pólvora, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:60, VMaxPes:60</t>
+          <t>Autopista Los Andes, Quillota, Quillota, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
         </is>
       </c>
       <c r="F31" s="12" t="n">
-        <v>100.6</v>
+        <v>73.3</v>
       </c>
       <c r="G31" s="12" t="n">
-        <v>147293.7</v>
+        <v>118470.6</v>
       </c>
       <c r="H31" s="12" t="n">
-        <v>395.6</v>
+        <v>80.90000000000001</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>GC TSVS-89 M AEDO</t>
         </is>
       </c>
       <c r="B32" s="12" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C32" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 11:32:00</t>
+          <t>2026/08/07 18:36:12</t>
         </is>
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>-33.066878,-71.63965</t>
+          <t>-33.06936,-71.36277</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
         <is>
-          <t>Camino La Pólvora, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:60, VMaxPes:60</t>
+          <t>Autopista Troncal Sur, Villa Alemana, Marga Marga, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
         </is>
       </c>
       <c r="F32" s="12" t="n">
-        <v>101.8</v>
+        <v>103.7</v>
       </c>
       <c r="G32" s="12" t="n">
-        <v>147293.8</v>
+        <v>118490.2</v>
       </c>
       <c r="H32" s="12" t="n">
-        <v>404.3</v>
+        <v>192.3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>GC TSVS-89 M AEDO</t>
         </is>
       </c>
       <c r="B33" s="12" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C33" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 11:32:04</t>
+          <t>2026/08/07 18:37:12</t>
         </is>
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
-          <t>-33.066455,-71.638545</t>
+          <t>-33.067906,-71.380727</t>
         </is>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>Camino La Pólvora, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:60, VMaxPes:60</t>
+          <t>Autopista Troncal Sur, Villa Alemana, Marga Marga, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
         </is>
       </c>
       <c r="F33" s="12" t="n">
         <v>103.6</v>
       </c>
       <c r="G33" s="12" t="n">
-        <v>147294</v>
+        <v>118491.9</v>
       </c>
       <c r="H33" s="12" t="n">
-        <v>410.7</v>
+        <v>177</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>GC TSVS-89 M AEDO</t>
         </is>
       </c>
       <c r="B34" s="12" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C34" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 11:32:17</t>
+          <t>2026/08/07 18:38:12</t>
         </is>
       </c>
       <c r="D34" s="15" t="inlineStr">
         <is>
-          <t>-33.066758,-71.634562</t>
+          <t>-33.066117,-71.397749</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
         <is>
-          <t>Camino La Pólvora, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:70, VMaxPes:70</t>
+          <t>Autopista Troncal Sur, Villa Alemana, Marga Marga, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
         </is>
       </c>
       <c r="F34" s="12" t="n">
-        <v>101</v>
+        <v>88.2</v>
       </c>
       <c r="G34" s="12" t="n">
-        <v>147294.3</v>
+        <v>118493.5</v>
       </c>
       <c r="H34" s="12" t="n">
-        <v>432.8</v>
+        <v>169.5</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>JAC  LYTS-17 G GALEA</t>
         </is>
       </c>
       <c r="B35" s="12" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>2026/08/01 11:32:53</t>
+          <t>2026/08/06 07:52:03</t>
         </is>
       </c>
       <c r="D35" s="15" t="inlineStr">
         <is>
-          <t>-33.072407,-71.627597</t>
+          <t>-32.680652,-71.425247</t>
         </is>
       </c>
       <c r="E35" s="12" t="inlineStr">
         <is>
-          <t>Camino La Pólvora, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:70, VMaxPes:70</t>
+          <t>Ruta E-30-F, Puchuncaví, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
         </is>
       </c>
       <c r="F35" s="12" t="n">
-        <v>85.90000000000001</v>
+        <v>101.1</v>
       </c>
       <c r="G35" s="12" t="n">
-        <v>147295.2</v>
+        <v>226852.1</v>
       </c>
       <c r="H35" s="12" t="n">
-        <v>431.9</v>
+        <v>88.7</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>GLP SKDX-44 V VIAL</t>
+          <t>JAC  LYTS-17 G GALEA</t>
         </is>
       </c>
       <c r="B36" s="12" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C36" s="12" t="inlineStr">
         <is>
-          <t>2026/08/02 12:14:56</t>
+          <t>2026/08/06 07:53:03</t>
         </is>
       </c>
       <c r="D36" s="15" t="inlineStr">
         <is>
-          <t>-33.09045,-71.541794</t>
+          <t>-32.670624,-71.425352</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
         <is>
-          <t>Ruta Las Palmas, Viña del Mar, Valparaíso, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
+          <t>Ruta E-30-F, Puchuncaví, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
         </is>
       </c>
       <c r="F36" s="12" t="n">
-        <v>102.2</v>
+        <v>63.9</v>
       </c>
       <c r="G36" s="12" t="n">
-        <v>147585.4</v>
+        <v>226853.2</v>
       </c>
       <c r="H36" s="12" t="n">
-        <v>321.6</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="7" t="inlineStr">
-        <is>
-          <t>GLP SKDX-44 V VIAL</t>
-        </is>
-      </c>
-      <c r="B37" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="C37" s="12" t="inlineStr">
-        <is>
-          <t>2026/08/02 12:15:15</t>
-        </is>
-      </c>
-      <c r="D37" s="15" t="inlineStr">
-        <is>
-          <t>-33.094806,-71.543443</t>
-        </is>
-      </c>
-      <c r="E37" s="12" t="inlineStr">
-        <is>
-          <t>Vía Las Palmas, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:80, VMaxPes:80</t>
-        </is>
-      </c>
-      <c r="F37" s="12" t="n">
-        <v>100.3</v>
-      </c>
-      <c r="G37" s="12" t="n">
-        <v>147586</v>
-      </c>
-      <c r="H37" s="12" t="n">
-        <v>318.4</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>GLP SKDX-44 V VIAL</t>
-        </is>
-      </c>
-      <c r="B38" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="C38" s="12" t="inlineStr">
-        <is>
-          <t>2026/08/02 12:15:30</t>
-        </is>
-      </c>
-      <c r="D38" s="15" t="inlineStr">
-        <is>
-          <t>-33.096963,-71.546855</t>
-        </is>
-      </c>
-      <c r="E38" s="12" t="inlineStr">
-        <is>
-          <t>s/n, Valparaíso, Valparaíso, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
-        </is>
-      </c>
-      <c r="F38" s="12" t="n">
-        <v>94.09999999999999</v>
-      </c>
-      <c r="G38" s="12" t="n">
-        <v>147586.4</v>
-      </c>
-      <c r="H38" s="12" t="n">
-        <v>321.6</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B39" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/27 06:25:04</t>
-        </is>
-      </c>
-      <c r="D39" s="15" t="inlineStr">
-        <is>
-          <t>-33.067327,-71.387599</t>
-        </is>
-      </c>
-      <c r="E39" s="12" t="inlineStr">
-        <is>
-          <t>Autopista Troncal Sur, Villa Alemana, Marga Marga, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
-        </is>
-      </c>
-      <c r="F39" s="12" t="n">
-        <v>104</v>
-      </c>
-      <c r="G39" s="12" t="n">
-        <v>115264</v>
-      </c>
-      <c r="H39" s="12" t="n">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B40" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C40" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/27 06:26:04</t>
-        </is>
-      </c>
-      <c r="D40" s="15" t="inlineStr">
-        <is>
-          <t>-33.068846,-71.370499</t>
-        </is>
-      </c>
-      <c r="E40" s="12" t="inlineStr">
-        <is>
-          <t>Autopista Troncal Sur, Villa Alemana, Marga Marga, Región de Valparaíso. VMaxLiv:120, VMaxPes:100</t>
-        </is>
-      </c>
-      <c r="F40" s="12" t="n">
-        <v>90.90000000000001</v>
-      </c>
-      <c r="G40" s="12" t="n">
-        <v>115265.6</v>
-      </c>
-      <c r="H40" s="12" t="n">
-        <v>176.9</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B41" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="C41" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/27 06:32:04</t>
-        </is>
-      </c>
-      <c r="D41" s="15" t="inlineStr">
-        <is>
-          <t>-33.016759,-71.31988</t>
-        </is>
-      </c>
-      <c r="E41" s="12" t="inlineStr">
-        <is>
-          <t>Autopista Los Andes, Limache, Marga Marga, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
-        </is>
-      </c>
-      <c r="F41" s="12" t="n">
-        <v>100.2</v>
-      </c>
-      <c r="G41" s="12" t="n">
-        <v>115274.5</v>
-      </c>
-      <c r="H41" s="12" t="n">
-        <v>108.7</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B42" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="C42" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/27 06:33:04</t>
-        </is>
-      </c>
-      <c r="D42" s="15" t="inlineStr">
-        <is>
-          <t>-33.004069,-71.328408</t>
-        </is>
-      </c>
-      <c r="E42" s="12" t="inlineStr">
-        <is>
-          <t>Autopista Los Andes, Limache, Marga Marga, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
-        </is>
-      </c>
-      <c r="F42" s="12" t="n">
-        <v>88.7</v>
-      </c>
-      <c r="G42" s="12" t="n">
-        <v>115276.1</v>
-      </c>
-      <c r="H42" s="12" t="n">
-        <v>96.59999999999999</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B43" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="C43" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/27 06:43:04</t>
-        </is>
-      </c>
-      <c r="D43" s="15" t="inlineStr">
-        <is>
-          <t>-32.911064,-71.269813</t>
-        </is>
-      </c>
-      <c r="E43" s="12" t="inlineStr">
-        <is>
-          <t>Autopista Los Andes, Quillota, Quillota, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
-        </is>
-      </c>
-      <c r="F43" s="12" t="n">
-        <v>100.4</v>
-      </c>
-      <c r="G43" s="12" t="n">
-        <v>115289.1</v>
-      </c>
-      <c r="H43" s="12" t="n">
-        <v>96.90000000000001</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B44" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="C44" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/27 06:44:04</t>
-        </is>
-      </c>
-      <c r="D44" s="15" t="inlineStr">
-        <is>
-          <t>-32.903617,-71.254498</t>
-        </is>
-      </c>
-      <c r="E44" s="12" t="inlineStr">
-        <is>
-          <t>Autopista Los Andes, Quillota, Quillota, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
-        </is>
-      </c>
-      <c r="F44" s="12" t="n">
-        <v>96.2</v>
-      </c>
-      <c r="G44" s="12" t="n">
-        <v>115290.8</v>
-      </c>
-      <c r="H44" s="12" t="n">
-        <v>105.4</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B45" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="C45" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/27 07:46:04</t>
-        </is>
-      </c>
-      <c r="D45" s="15" t="inlineStr">
-        <is>
-          <t>-32.572429,-71.289271</t>
-        </is>
-      </c>
-      <c r="E45" s="12" t="inlineStr">
-        <is>
-          <t>Ruta E-462, Zapallar, Petorca, Región de Valparaíso. VMaxLiv:60, VMaxPes:60</t>
-        </is>
-      </c>
-      <c r="F45" s="12" t="n">
-        <v>101.5</v>
-      </c>
-      <c r="G45" s="12" t="n">
-        <v>115358.6</v>
-      </c>
-      <c r="H45" s="12" t="n">
-        <v>82.5</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B46" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="C46" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/27 07:47:04</t>
-        </is>
-      </c>
-      <c r="D46" s="15" t="inlineStr">
-        <is>
-          <t>-32.569254,-71.276721</t>
-        </is>
-      </c>
-      <c r="E46" s="12" t="inlineStr">
-        <is>
-          <t>Ruta E-462, Zapallar, Petorca, Región de Valparaíso. VMaxLiv:60, VMaxPes:60</t>
-        </is>
-      </c>
-      <c r="F46" s="12" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="G46" s="12" t="n">
-        <v>115359.8</v>
-      </c>
-      <c r="H46" s="12" t="n">
-        <v>96.3</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B47" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="C47" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/27 07:50:04</t>
-        </is>
-      </c>
-      <c r="D47" s="15" t="inlineStr">
-        <is>
-          <t>-32.549855,-71.268268</t>
-        </is>
-      </c>
-      <c r="E47" s="12" t="inlineStr">
-        <is>
-          <t>Ruta 5 Norte, Zapallar, Petorca, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
-        </is>
-      </c>
-      <c r="F47" s="12" t="n">
-        <v>103.1</v>
-      </c>
-      <c r="G47" s="12" t="n">
-        <v>115363.5</v>
-      </c>
-      <c r="H47" s="12" t="n">
-        <v>107.9</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B48" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="C48" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/27 07:51:04</t>
-        </is>
-      </c>
-      <c r="D48" s="15" t="inlineStr">
-        <is>
-          <t>-32.534791,-71.264781</t>
-        </is>
-      </c>
-      <c r="E48" s="12" t="inlineStr">
-        <is>
-          <t>Ruta 5 Norte, Zapallar, Petorca, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
-        </is>
-      </c>
-      <c r="F48" s="12" t="n">
-        <v>102</v>
-      </c>
-      <c r="G48" s="12" t="n">
-        <v>115365.2</v>
-      </c>
-      <c r="H48" s="12" t="n">
-        <v>114.7</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B49" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="C49" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/27 07:52:04</t>
-        </is>
-      </c>
-      <c r="D49" s="15" t="inlineStr">
-        <is>
-          <t>-32.519725,-71.261213</t>
-        </is>
-      </c>
-      <c r="E49" s="12" t="inlineStr">
-        <is>
-          <t>Ruta 5 Norte, La Ligua, Petorca, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
-        </is>
-      </c>
-      <c r="F49" s="12" t="n">
-        <v>100.7</v>
-      </c>
-      <c r="G49" s="12" t="n">
-        <v>115366.9</v>
-      </c>
-      <c r="H49" s="12" t="n">
-        <v>101.1</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B50" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="C50" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/27 07:53:04</t>
-        </is>
-      </c>
-      <c r="D50" s="15" t="inlineStr">
-        <is>
-          <t>-32.506255,-71.259684</t>
-        </is>
-      </c>
-      <c r="E50" s="12" t="inlineStr">
-        <is>
-          <t>Ruta 5 Norte, La Ligua, Petorca, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
-        </is>
-      </c>
-      <c r="F50" s="12" t="n">
-        <v>89.3</v>
-      </c>
-      <c r="G50" s="12" t="n">
-        <v>115368.4</v>
-      </c>
-      <c r="H50" s="12" t="n">
-        <v>77.7</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B51" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="C51" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/31 19:07:11</t>
-        </is>
-      </c>
-      <c r="D51" s="15" t="inlineStr">
-        <is>
-          <t>-32.870929,-71.229809</t>
-        </is>
-      </c>
-      <c r="E51" s="12" t="inlineStr">
-        <is>
-          <t>Autopista Los Andes, Quillota, Quillota, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
-        </is>
-      </c>
-      <c r="F51" s="12" t="n">
-        <v>101.9</v>
-      </c>
-      <c r="G51" s="12" t="n">
-        <v>116983.2</v>
-      </c>
-      <c r="H51" s="12" t="n">
-        <v>126.4</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B52" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="C52" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/31 19:08:11</t>
-        </is>
-      </c>
-      <c r="D52" s="15" t="inlineStr">
-        <is>
-          <t>-32.885976,-71.232073</t>
-        </is>
-      </c>
-      <c r="E52" s="12" t="inlineStr">
-        <is>
-          <t>Autopista Los Andes, Quillota, Quillota, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
-        </is>
-      </c>
-      <c r="F52" s="12" t="n">
-        <v>102.4</v>
-      </c>
-      <c r="G52" s="12" t="n">
-        <v>116984.9</v>
-      </c>
-      <c r="H52" s="12" t="n">
-        <v>117.9</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B53" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="C53" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/31 19:09:11</t>
-        </is>
-      </c>
-      <c r="D53" s="15" t="inlineStr">
-        <is>
-          <t>-32.898972,-71.239656</t>
-        </is>
-      </c>
-      <c r="E53" s="12" t="inlineStr">
-        <is>
-          <t>Autopista Los Andes, Quillota, Quillota, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
-        </is>
-      </c>
-      <c r="F53" s="12" t="n">
-        <v>97.40000000000001</v>
-      </c>
-      <c r="G53" s="12" t="n">
-        <v>116986.6</v>
-      </c>
-      <c r="H53" s="12" t="n">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B54" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="C54" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/31 19:10:11</t>
-        </is>
-      </c>
-      <c r="D54" s="15" t="inlineStr">
-        <is>
-          <t>-32.904194,-71.25627</t>
-        </is>
-      </c>
-      <c r="E54" s="12" t="inlineStr">
-        <is>
-          <t>Autopista Los Andes, Quillota, Quillota, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
-        </is>
-      </c>
-      <c r="F54" s="12" t="n">
-        <v>100.9</v>
-      </c>
-      <c r="G54" s="12" t="n">
-        <v>116988.3</v>
-      </c>
-      <c r="H54" s="12" t="n">
-        <v>100.9</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B55" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="C55" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/31 19:11:11</t>
-        </is>
-      </c>
-      <c r="D55" s="15" t="inlineStr">
-        <is>
-          <t>-32.912396,-71.271115</t>
-        </is>
-      </c>
-      <c r="E55" s="12" t="inlineStr">
-        <is>
-          <t>Autopista Los Andes, Quillota, Quillota, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
-        </is>
-      </c>
-      <c r="F55" s="12" t="n">
-        <v>102.5</v>
-      </c>
-      <c r="G55" s="12" t="n">
-        <v>116990</v>
-      </c>
-      <c r="H55" s="12" t="n">
-        <v>91.09999999999999</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B56" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="C56" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/31 19:12:11</t>
-        </is>
-      </c>
-      <c r="D56" s="15" t="inlineStr">
-        <is>
-          <t>-32.924905,-71.281892</t>
-        </is>
-      </c>
-      <c r="E56" s="12" t="inlineStr">
-        <is>
-          <t>Autopista Los Andes, Quillota, Quillota, Región de Valparaíso. VMaxLiv:100, VMaxPes:90</t>
-        </is>
-      </c>
-      <c r="F56" s="12" t="n">
-        <v>100.7</v>
-      </c>
-      <c r="G56" s="12" t="n">
-        <v>116991.7</v>
-      </c>
-      <c r="H56" s="12" t="n">
-        <v>81.3</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="7" t="inlineStr">
-        <is>
-          <t>GC TSVS-89 M AEDO</t>
-        </is>
-      </c>
-      <c r="B57" s="12" t="n">
-        <v>7</v>
-      </c>
-      <c r="C57" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/31 19:12:55</t>
-        </is>
-      </c>
-      <c r="D57" s="15" t="inlineStr">
-        <is>
-          <t>-32.933783,-71.288593</t>
-        </is>
-      </c>
-      <c r="E57" s="12" t="inlineStr">
-        <is>
-          <t>Autopista Los Andes, Quillota, Quillota, Región de Valparaíso. VMaxLiv:50, VMaxPes:50</t>
-        </is>
-      </c>
-      <c r="F57" s="12" t="n">
-        <v>68.8</v>
-      </c>
-      <c r="G57" s="12" t="n">
-        <v>116992.9</v>
-      </c>
-      <c r="H57" s="12" t="n">
-        <v>76.90000000000001</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="7" t="inlineStr">
-        <is>
-          <t>GC MAXUS PCRF-25 TERRENO</t>
-        </is>
-      </c>
-      <c r="B58" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C58" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/31 14:57:40</t>
-        </is>
-      </c>
-      <c r="D58" s="15" t="inlineStr">
-        <is>
-          <t>-32.577562,-71.309168</t>
-        </is>
-      </c>
-      <c r="E58" s="12" t="inlineStr">
-        <is>
-          <t>Ruta E-462, Zapallar, Petorca, Región de Valparaíso. VMaxLiv:60, VMaxPes:60</t>
-        </is>
-      </c>
-      <c r="F58" s="12" t="n">
-        <v>100.4</v>
-      </c>
-      <c r="G58" s="12" t="n">
-        <v>90949.10000000001</v>
-      </c>
-      <c r="H58" s="12" t="n">
-        <v>67.5</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="7" t="inlineStr">
-        <is>
-          <t>GC MAXUS PCRF-25 TERRENO</t>
-        </is>
-      </c>
-      <c r="B59" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="C59" s="12" t="inlineStr">
-        <is>
-          <t>2026/07/31 14:58:40</t>
-        </is>
-      </c>
-      <c r="D59" s="15" t="inlineStr">
-        <is>
-          <t>-32.583363,-71.323384</t>
-        </is>
-      </c>
-      <c r="E59" s="12" t="inlineStr">
-        <is>
-          <t>Ruta E-462, Zapallar, Petorca, Región de Valparaíso. VMaxLiv:60, VMaxPes:60</t>
-        </is>
-      </c>
-      <c r="F59" s="12" t="n">
-        <v>91.59999999999999</v>
-      </c>
-      <c r="G59" s="12" t="n">
-        <v>90950.60000000001</v>
-      </c>
-      <c r="H59" s="12" t="n">
-        <v>66.90000000000001</v>
+        <v>110.3</v>
       </c>
     </row>
   </sheetData>
@@ -9898,35 +11014,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId54"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <pageSetup orientation="default" paperSize="1" scale="100" pageOrder="downThenOver" blackAndWhite="0" draft="0" errors="displayed"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId55"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId32"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>